<commit_message>
updated the ui version 2
</commit_message>
<xml_diff>
--- a/docs/mini-project-report/QRSathi_Requirement_Traceability_Matrix.xlsx
+++ b/docs/mini-project-report/QRSathi_Requirement_Traceability_Matrix.xlsx
@@ -3237,349 +3237,349 @@
     <t>/api/admin/auth/login</t>
   </si>
   <si>
+    <t>rate-limited</t>
+  </si>
+  <si>
+    <t>Admin sign-in step 1 (password); returns MFA ticket when MFA enabled</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/auth/login/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/auth/logout</t>
+  </si>
+  <si>
+    <t>admin session (checked in handler)</t>
+  </si>
+  <si>
+    <t>End admin-console session</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/auth/logout/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/auth/me</t>
+  </si>
+  <si>
+    <t>Current administrator</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/auth/me/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/auth/mfa</t>
+  </si>
+  <si>
+    <t>Admin sign-in step 2 (TOTP or recovery code)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/auth/mfa/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/auth/reauth</t>
+  </si>
+  <si>
+    <t>admin session (checked in handler), rate-limited</t>
+  </si>
+  <si>
+    <t>Re-confirm password (+TOTP) for sensitive actions</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/auth/reauth/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/branding</t>
+  </si>
+  <si>
+    <t>GET, PUT, POST</t>
+  </si>
+  <si>
+    <t>admin, rate-limited</t>
+  </si>
+  <si>
+    <t>GET branding state; PUT draft; POST publish / discard / reset</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/branding/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/branding/assets</t>
+  </si>
+  <si>
+    <t>Upload logo/favicon/social image (validated)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/branding/assets/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/catalog</t>
+  </si>
+  <si>
+    <t>Products and barcodes overview (admin)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/catalog/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/email</t>
+  </si>
+  <si>
+    <t>GET, POST</t>
+  </si>
+  <si>
+    <t>GET SMTP status (no credentials); POST test mail to own address</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/email/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/logs</t>
+  </si>
+  <si>
+    <t>System log entries</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/logs/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/mfa</t>
+  </si>
+  <si>
+    <t>admin (MFA not required), rate-limited</t>
+  </si>
+  <si>
+    <t>GET MFA status; POST setup / enable / disable / regenerate recovery codes</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/mfa/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/payments</t>
+  </si>
+  <si>
+    <t>Payment records</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/payments/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/payments/config</t>
+  </si>
+  <si>
+    <t>GET, PUT, PATCH, POST</t>
+  </si>
+  <si>
+    <t>admin, super admin, recent re-auth (super admin), rate-limited</t>
+  </si>
+  <si>
+    <t>GET gateway status (never secrets); PUT credentials (super admin + re-auth); PATCH enable/mode; POST verify</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/payments/config/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/plans</t>
+  </si>
+  <si>
+    <t>admin, super admin, rate-limited</t>
+  </si>
+  <si>
+    <t>GET plans; POST create plan (super admin)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/plans/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/plans/[id]</t>
+  </si>
+  <si>
+    <t>PATCH, POST</t>
+  </si>
+  <si>
+    <t>super admin, rate-limited</t>
+  </si>
+  <si>
+    <t>PATCH edit plan (confirm if live subscribers); POST action: duplicate, publish, unpublish, archive, restore or sync provider plans</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/plans/[id]/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/plans/reorder</t>
+  </si>
+  <si>
+    <t>super admin</t>
+  </si>
+  <si>
+    <t>Reorder plans (super admin)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/plans/reorder/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/qrcodes</t>
+  </si>
+  <si>
+    <t>List dynamic and hosted QR codes</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/qrcodes/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/qrcodes/[id]</t>
+  </si>
+  <si>
+    <t>PATCH, DELETE</t>
+  </si>
+  <si>
+    <t>PATCH status active/paused/disabled; DELETE QR code</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/qrcodes/[id]/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/reports</t>
+  </si>
+  <si>
+    <t>List abuse reports</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/reports/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/reports/[id]</t>
+  </si>
+  <si>
+    <t>PATCH</t>
+  </si>
+  <si>
+    <t>PATCH report status: open, resolved or dismissed (audited)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/reports/[id]/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/security</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/security/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/settings</t>
+  </si>
+  <si>
+    <t>GET, PUT</t>
+  </si>
+  <si>
+    <t>GET/PUT general settings</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/settings/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/stats</t>
+  </si>
+  <si>
+    <t>Overview statistics</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/stats/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/subscriptions</t>
+  </si>
+  <si>
+    <t>List subscriptions</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/subscriptions/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/subscriptions/[id]</t>
+  </si>
+  <si>
+    <t>Cancel a subscription (super admin)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/subscriptions/[id]/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/system</t>
+  </si>
+  <si>
+    <t>Configuration and health status</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/system/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/users</t>
+  </si>
+  <si>
+    <t>Search and page users (no secrets)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/users/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/users/[id]</t>
+  </si>
+  <si>
+    <t>PATCH, POST, DELETE</t>
+  </si>
+  <si>
+    <t>admin, super admin</t>
+  </si>
+  <si>
+    <t>PATCH role/plan/status; POST revoke sessions / send reset; DELETE account (super admin)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/users/[id]/route.ts</t>
+  </si>
+  <si>
+    <t>/api/admin/users/bulk</t>
+  </si>
+  <si>
+    <t>Bulk suspend / reactivate / revoke sessions (≤100 ids)</t>
+  </si>
+  <si>
+    <t>src/app/api/admin/users/bulk/route.ts</t>
+  </si>
+  <si>
+    <t>/api/analytics</t>
+  </si>
+  <si>
+    <t>Scan statistics limited to plan's analyticsDays</t>
+  </si>
+  <si>
+    <t>src/app/api/analytics/route.ts</t>
+  </si>
+  <si>
+    <t>/api/analytics/export</t>
+  </si>
+  <si>
+    <t>user, plan feature</t>
+  </si>
+  <si>
+    <t>CSV export of scans (requires analyticsExport feature)</t>
+  </si>
+  <si>
+    <t>src/app/api/analytics/export/route.ts</t>
+  </si>
+  <si>
+    <t>/api/auth/forgot</t>
+  </si>
+  <si>
+    <t>Request password-reset e-mail (same response for any e-mail)</t>
+  </si>
+  <si>
+    <t>src/app/api/auth/forgot/route.ts</t>
+  </si>
+  <si>
+    <t>/api/auth/google</t>
+  </si>
+  <si>
     <t>public</t>
-  </si>
-  <si>
-    <t>Admin sign-in step 1 (password); returns MFA ticket when MFA enabled</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/auth/login/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/auth/logout</t>
-  </si>
-  <si>
-    <t>admin session (checked in handler)</t>
-  </si>
-  <si>
-    <t>End admin-console session</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/auth/logout/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/auth/me</t>
-  </si>
-  <si>
-    <t>Current administrator</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/auth/me/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/auth/mfa</t>
-  </si>
-  <si>
-    <t>rate-limited</t>
-  </si>
-  <si>
-    <t>Admin sign-in step 2 (TOTP or recovery code)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/auth/mfa/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/auth/reauth</t>
-  </si>
-  <si>
-    <t>admin session (checked in handler), rate-limited</t>
-  </si>
-  <si>
-    <t>Re-confirm password (+TOTP) for sensitive actions</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/auth/reauth/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/branding</t>
-  </si>
-  <si>
-    <t>GET, PUT, POST</t>
-  </si>
-  <si>
-    <t>admin, rate-limited</t>
-  </si>
-  <si>
-    <t>GET branding state; PUT draft; POST publish / discard / reset</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/branding/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/branding/assets</t>
-  </si>
-  <si>
-    <t>Upload logo/favicon/social image (validated)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/branding/assets/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/catalog</t>
-  </si>
-  <si>
-    <t>Products and barcodes overview (admin)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/catalog/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/email</t>
-  </si>
-  <si>
-    <t>GET, POST</t>
-  </si>
-  <si>
-    <t>GET SMTP status (no credentials); POST test mail to own address</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/email/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/logs</t>
-  </si>
-  <si>
-    <t>System log entries</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/logs/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/mfa</t>
-  </si>
-  <si>
-    <t>admin (MFA not required), rate-limited</t>
-  </si>
-  <si>
-    <t>GET MFA status; POST setup / enable / disable / regenerate recovery codes</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/mfa/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/payments</t>
-  </si>
-  <si>
-    <t>Payment records</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/payments/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/payments/config</t>
-  </si>
-  <si>
-    <t>GET, PUT, PATCH, POST</t>
-  </si>
-  <si>
-    <t>admin, super admin, recent re-auth (super admin), rate-limited</t>
-  </si>
-  <si>
-    <t>GET gateway status (never secrets); PUT credentials (super admin + re-auth); PATCH enable/mode; POST verify</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/payments/config/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/plans</t>
-  </si>
-  <si>
-    <t>admin, super admin, rate-limited</t>
-  </si>
-  <si>
-    <t>GET plans; POST create plan (super admin)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/plans/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/plans/[id]</t>
-  </si>
-  <si>
-    <t>PATCH, POST</t>
-  </si>
-  <si>
-    <t>super admin, rate-limited</t>
-  </si>
-  <si>
-    <t>PATCH edit plan (confirm if live subscribers); POST action: duplicate, publish, unpublish, archive, restore or sync provider plans</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/plans/[id]/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/plans/reorder</t>
-  </si>
-  <si>
-    <t>super admin</t>
-  </si>
-  <si>
-    <t>Reorder plans (super admin)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/plans/reorder/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/qrcodes</t>
-  </si>
-  <si>
-    <t>List dynamic and hosted QR codes</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/qrcodes/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/qrcodes/[id]</t>
-  </si>
-  <si>
-    <t>PATCH, DELETE</t>
-  </si>
-  <si>
-    <t>PATCH status active/paused/disabled; DELETE QR code</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/qrcodes/[id]/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/reports</t>
-  </si>
-  <si>
-    <t>List abuse reports</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/reports/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/reports/[id]</t>
-  </si>
-  <si>
-    <t>PATCH</t>
-  </si>
-  <si>
-    <t>PATCH report status: open, resolved or dismissed (audited)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/reports/[id]/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/security</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/security/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/settings</t>
-  </si>
-  <si>
-    <t>GET, PUT</t>
-  </si>
-  <si>
-    <t>GET/PUT general settings</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/settings/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/stats</t>
-  </si>
-  <si>
-    <t>Overview statistics</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/stats/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/subscriptions</t>
-  </si>
-  <si>
-    <t>List subscriptions</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/subscriptions/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/subscriptions/[id]</t>
-  </si>
-  <si>
-    <t>Cancel a subscription (super admin)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/subscriptions/[id]/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/system</t>
-  </si>
-  <si>
-    <t>Configuration and health status</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/system/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/users</t>
-  </si>
-  <si>
-    <t>Search and page users (no secrets)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/users/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/users/[id]</t>
-  </si>
-  <si>
-    <t>PATCH, POST, DELETE</t>
-  </si>
-  <si>
-    <t>admin, super admin</t>
-  </si>
-  <si>
-    <t>PATCH role/plan/status; POST revoke sessions / send reset; DELETE account (super admin)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/users/[id]/route.ts</t>
-  </si>
-  <si>
-    <t>/api/admin/users/bulk</t>
-  </si>
-  <si>
-    <t>Bulk suspend / reactivate / revoke sessions (≤100 ids)</t>
-  </si>
-  <si>
-    <t>src/app/api/admin/users/bulk/route.ts</t>
-  </si>
-  <si>
-    <t>/api/analytics</t>
-  </si>
-  <si>
-    <t>Scan statistics limited to plan's analyticsDays</t>
-  </si>
-  <si>
-    <t>src/app/api/analytics/route.ts</t>
-  </si>
-  <si>
-    <t>/api/analytics/export</t>
-  </si>
-  <si>
-    <t>user, plan feature</t>
-  </si>
-  <si>
-    <t>CSV export of scans (requires analyticsExport feature)</t>
-  </si>
-  <si>
-    <t>src/app/api/analytics/export/route.ts</t>
-  </si>
-  <si>
-    <t>/api/auth/forgot</t>
-  </si>
-  <si>
-    <t>Request password-reset e-mail (same response for any e-mail)</t>
-  </si>
-  <si>
-    <t>src/app/api/auth/forgot/route.ts</t>
-  </si>
-  <si>
-    <t>/api/auth/google</t>
   </si>
   <si>
     <t>Start Google OAuth flow</t>
@@ -9598,69 +9598,69 @@
         <v>1062</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>1083</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>1084</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>1085</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>1062</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>1087</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>1088</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>1089</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>1090</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>1091</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>1092</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>1093</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>1094</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>1062</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>1095</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>1096</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>1097</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>1067</v>
@@ -9669,32 +9669,32 @@
         <v>1068</v>
       </c>
       <c r="D12" s="3" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>1099</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>1100</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>1101</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="3" t="s">
+        <v>1091</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>1102</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>1092</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>1103</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>1104</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>1067</v>
@@ -9703,32 +9703,32 @@
         <v>1068</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>1106</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>1107</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>1108</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>1102</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>1109</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>1110</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>1111</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>1067</v>
@@ -9737,83 +9737,83 @@
         <v>1068</v>
       </c>
       <c r="D16" s="3" t="s">
+        <v>1112</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>1113</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>1114</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>1115</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>1116</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>1117</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>1118</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>1119</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>1120</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>1102</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>1121</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>1122</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>1123</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>1124</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>1125</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>1126</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>1127</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>1128</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>1062</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>1129</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>1130</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>1131</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>1132</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>1067</v>
@@ -9822,32 +9822,32 @@
         <v>1068</v>
       </c>
       <c r="D21" s="3" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>1134</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>1135</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>1136</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>1137</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>1068</v>
       </c>
       <c r="D22" s="3" t="s">
+        <v>1137</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>1138</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>1139</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>1067</v>
@@ -9856,32 +9856,32 @@
         <v>1068</v>
       </c>
       <c r="D23" s="3" t="s">
+        <v>1140</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>1141</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>1142</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>1143</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>1144</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>1068</v>
       </c>
       <c r="D24" s="3" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>1145</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>1146</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>1067</v>
@@ -9893,29 +9893,29 @@
         <v>964</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>1149</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="C26" s="3" t="s">
+        <v>1091</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>1150</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>1092</v>
-      </c>
-      <c r="D26" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>1151</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>1152</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>1067</v>
@@ -9924,15 +9924,15 @@
         <v>1068</v>
       </c>
       <c r="D27" s="3" t="s">
+        <v>1153</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>1154</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>1155</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>1067</v>
@@ -9941,32 +9941,32 @@
         <v>1068</v>
       </c>
       <c r="D28" s="3" t="s">
+        <v>1156</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>1157</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>1158</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>1062</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D29" s="3" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>1160</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>1161</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>1067</v>
@@ -9975,15 +9975,15 @@
         <v>1068</v>
       </c>
       <c r="D30" s="3" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>1163</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>1164</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>1067</v>
@@ -9992,32 +9992,32 @@
         <v>1068</v>
       </c>
       <c r="D31" s="3" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>1166</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>1167</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>1168</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="C32" s="3" t="s">
         <v>1169</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="D32" s="3" t="s">
         <v>1170</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="E32" s="3" t="s">
         <v>1171</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>1172</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>1062</v>
@@ -10026,15 +10026,15 @@
         <v>1068</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>1174</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>1175</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>1067</v>
@@ -10043,55 +10043,55 @@
         <v>1063</v>
       </c>
       <c r="D34" s="3" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>1177</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>1067</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>1179</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>1180</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>1181</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>1182</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>1062</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>1083</v>
+        <v>1072</v>
       </c>
       <c r="D36" s="3" t="s">
+        <v>1183</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>1184</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>1185</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>1067</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>1072</v>
+        <v>1186</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>1187</v>
@@ -10108,7 +10108,7 @@
         <v>1067</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>1072</v>
+        <v>1186</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>1190</v>
@@ -10142,7 +10142,7 @@
         <v>1062</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>1072</v>
+        <v>1186</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>1196</v>
@@ -10176,7 +10176,7 @@
         <v>1062</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>1083</v>
+        <v>1072</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>1203</v>
@@ -10193,7 +10193,7 @@
         <v>1062</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>1083</v>
+        <v>1072</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>1206</v>
@@ -10329,7 +10329,7 @@
         <v>1067</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>1072</v>
+        <v>1186</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>1231</v>
@@ -10377,7 +10377,7 @@
         <v>1239</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>1063</v>
@@ -10496,7 +10496,7 @@
         <v>1260</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>1058</v>
@@ -10550,7 +10550,7 @@
         <v>1062</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>1083</v>
+        <v>1072</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>1270</v>
@@ -10584,7 +10584,7 @@
         <v>1067</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>1072</v>
+        <v>1186</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>1276</v>
@@ -10601,7 +10601,7 @@
         <v>1067</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>1072</v>
+        <v>1186</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>1279</v>
@@ -10618,7 +10618,7 @@
         <v>1067</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>1072</v>
+        <v>1186</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>1282</v>

</xml_diff>